<commit_message>
revise code for library report diagram
</commit_message>
<xml_diff>
--- a/data_raw/OS-Inventory-list-20260518.xlsx
+++ b/data_raw/OS-Inventory-list-20260518.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xiuqili/Documents/GitHub/Open-Science-Inventory/data_raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3DDB1E8-DD06-094B-BCCC-BF02AFD0C897}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78BB41AB-6F2D-F44F-B55B-A71285221401}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16320" yWindow="4980" windowWidth="35380" windowHeight="21580" xr2:uid="{1509BDA8-4FD2-7641-BB7D-D0BB426F409D}"/>
+    <workbookView xWindow="2280" yWindow="2400" windowWidth="41000" windowHeight="25360" xr2:uid="{1509BDA8-4FD2-7641-BB7D-D0BB426F409D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="103">
   <si>
     <t>Category</t>
   </si>
@@ -338,6 +338,12 @@
   </si>
   <si>
     <t>Data Source Access Review</t>
+  </si>
+  <si>
+    <t>Color</t>
+  </si>
+  <si>
+    <t>Review</t>
   </si>
 </sst>
 </file>
@@ -780,7 +786,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20BAB806-8A7F-5D43-B5BC-96EB20C6A4E4}">
-  <dimension ref="A1:G56"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.6640625" bestFit="1" customWidth="1"/>
@@ -790,9 +796,10 @@
     <col min="5" max="5" width="24" customWidth="1"/>
     <col min="6" max="6" width="23" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="29.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -814,8 +821,11 @@
       <c r="G1" s="1" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H1" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="11" t="s">
         <v>22</v>
       </c>
@@ -829,8 +839,11 @@
       <c r="E2" s="11"/>
       <c r="F2" s="11"/>
       <c r="G2" s="11"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H2" s="12" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="11" t="s">
         <v>22</v>
       </c>
@@ -844,8 +857,11 @@
       <c r="E3" s="11"/>
       <c r="F3" s="11"/>
       <c r="G3" s="11"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H3" s="12" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="11" t="s">
         <v>22</v>
       </c>
@@ -859,8 +875,11 @@
       <c r="E4" s="11"/>
       <c r="F4" s="11"/>
       <c r="G4" s="11"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H4" s="12" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" s="11" t="s">
         <v>22</v>
       </c>
@@ -874,8 +893,11 @@
       <c r="E5" s="11"/>
       <c r="F5" s="11"/>
       <c r="G5" s="11"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H5" s="12" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="11" t="s">
         <v>22</v>
       </c>
@@ -889,8 +911,11 @@
       <c r="E6" s="11"/>
       <c r="F6" s="11"/>
       <c r="G6" s="11"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H6" s="12" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="11" t="s">
         <v>22</v>
       </c>
@@ -904,8 +929,11 @@
       <c r="E7" s="11"/>
       <c r="F7" s="11"/>
       <c r="G7" s="11"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H7" s="12" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" s="11" t="s">
         <v>22</v>
       </c>
@@ -919,8 +947,11 @@
       <c r="E8" s="11"/>
       <c r="F8" s="11"/>
       <c r="G8" s="11"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H8" s="12" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
         <v>30</v>
       </c>
@@ -936,8 +967,9 @@
       </c>
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H9" s="4"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
         <v>30</v>
       </c>
@@ -953,8 +985,9 @@
       </c>
       <c r="F10" s="3"/>
       <c r="G10" s="3"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H10" s="4"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
         <v>30</v>
       </c>
@@ -970,8 +1003,9 @@
       </c>
       <c r="F11" s="3"/>
       <c r="G11" s="3"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H11" s="4"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
         <v>30</v>
       </c>
@@ -987,8 +1021,9 @@
       </c>
       <c r="F12" s="3"/>
       <c r="G12" s="3"/>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H12" s="4"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
         <v>30</v>
       </c>
@@ -1004,8 +1039,9 @@
       </c>
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H13" s="4"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
         <v>30</v>
       </c>
@@ -1021,8 +1057,9 @@
       </c>
       <c r="F14" s="3"/>
       <c r="G14" s="3"/>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H14" s="4"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
         <v>30</v>
       </c>
@@ -1038,8 +1075,9 @@
       </c>
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H15" s="4"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" s="7" t="s">
         <v>34</v>
       </c>
@@ -1059,8 +1097,11 @@
         <v>51</v>
       </c>
       <c r="G16" s="7"/>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H16" s="8" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" s="7" t="s">
         <v>34</v>
       </c>
@@ -1080,8 +1121,11 @@
         <v>51</v>
       </c>
       <c r="G17" s="7"/>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H17" s="8" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" s="7" t="s">
         <v>34</v>
       </c>
@@ -1101,8 +1145,11 @@
         <v>8</v>
       </c>
       <c r="G18" s="7"/>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H18" s="8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" s="7" t="s">
         <v>34</v>
       </c>
@@ -1122,8 +1169,11 @@
         <v>8</v>
       </c>
       <c r="G19" s="7"/>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H19" s="8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" s="7" t="s">
         <v>34</v>
       </c>
@@ -1143,8 +1193,11 @@
         <v>8</v>
       </c>
       <c r="G20" s="7"/>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H20" s="8" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" s="7" t="s">
         <v>34</v>
       </c>
@@ -1164,8 +1217,11 @@
         <v>8</v>
       </c>
       <c r="G21" s="7"/>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H21" s="8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="7" t="s">
         <v>34</v>
       </c>
@@ -1185,8 +1241,11 @@
         <v>8</v>
       </c>
       <c r="G22" s="7"/>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H22" s="8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" s="7" t="s">
         <v>34</v>
       </c>
@@ -1206,8 +1265,11 @@
         <v>31</v>
       </c>
       <c r="G23" s="7"/>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H23" s="8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" s="7" t="s">
         <v>34</v>
       </c>
@@ -1227,8 +1289,11 @@
         <v>8</v>
       </c>
       <c r="G24" s="7"/>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H24" s="8" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" s="7" t="s">
         <v>34</v>
       </c>
@@ -1248,8 +1313,11 @@
         <v>92</v>
       </c>
       <c r="G25" s="7"/>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H25" s="8" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A26" s="7" t="s">
         <v>34</v>
       </c>
@@ -1269,8 +1337,11 @@
         <v>31</v>
       </c>
       <c r="G26" s="7"/>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H26" s="8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27" s="7" t="s">
         <v>34</v>
       </c>
@@ -1290,8 +1361,11 @@
         <v>7</v>
       </c>
       <c r="G27" s="7"/>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H27" s="8" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A28" s="7" t="s">
         <v>34</v>
       </c>
@@ -1311,8 +1385,11 @@
         <v>8</v>
       </c>
       <c r="G28" s="7"/>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H28" s="8" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A29" s="7" t="s">
         <v>34</v>
       </c>
@@ -1332,8 +1409,11 @@
         <v>8</v>
       </c>
       <c r="G29" s="7"/>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H29" s="8" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A30" s="7" t="s">
         <v>34</v>
       </c>
@@ -1353,8 +1433,11 @@
         <v>8</v>
       </c>
       <c r="G30" s="7"/>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H30" s="8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" s="7" t="s">
         <v>34</v>
       </c>
@@ -1374,8 +1457,11 @@
         <v>8</v>
       </c>
       <c r="G31" s="7"/>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H31" s="8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32" s="7" t="s">
         <v>34</v>
       </c>
@@ -1395,8 +1481,11 @@
         <v>31</v>
       </c>
       <c r="G32" s="7"/>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H32" s="8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33" s="5" t="s">
         <v>41</v>
       </c>
@@ -1416,8 +1505,11 @@
         <v>33</v>
       </c>
       <c r="G33" s="5"/>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H33" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A34" s="5" t="s">
         <v>41</v>
       </c>
@@ -1439,8 +1531,11 @@
       <c r="G34" s="5" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H34" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A35" s="5" t="s">
         <v>41</v>
       </c>
@@ -1462,8 +1557,11 @@
       <c r="G35" s="5" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H35" s="6" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A36" s="5" t="s">
         <v>41</v>
       </c>
@@ -1485,8 +1583,11 @@
       <c r="G36" s="5" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H36" s="6" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A37" s="5" t="s">
         <v>41</v>
       </c>
@@ -1508,8 +1609,11 @@
       <c r="G37" s="5" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H37" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A38" s="5" t="s">
         <v>41</v>
       </c>
@@ -1531,8 +1635,11 @@
       <c r="G38" s="5" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H38" s="6" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A39" s="5" t="s">
         <v>41</v>
       </c>
@@ -1554,8 +1661,11 @@
       <c r="G39" s="5" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H39" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" s="5" t="s">
         <v>41</v>
       </c>
@@ -1577,8 +1687,11 @@
       <c r="G40" s="5" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H40" s="6" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A41" s="5" t="s">
         <v>41</v>
       </c>
@@ -1600,8 +1713,11 @@
       <c r="G41" s="5" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H41" s="6" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A42" s="5" t="s">
         <v>41</v>
       </c>
@@ -1623,8 +1739,11 @@
       <c r="G42" s="5" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H42" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A43" s="5" t="s">
         <v>41</v>
       </c>
@@ -1646,8 +1765,11 @@
       <c r="G43" s="5" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H43" s="6" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A44" s="5" t="s">
         <v>41</v>
       </c>
@@ -1669,8 +1791,11 @@
       <c r="G44" s="5" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H44" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A45" s="5" t="s">
         <v>41</v>
       </c>
@@ -1692,8 +1817,11 @@
       <c r="G45" s="5" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H45" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A46" s="9" t="s">
         <v>99</v>
       </c>
@@ -1715,8 +1843,11 @@
       <c r="G46" s="9" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H46" s="10" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A47" s="9" t="s">
         <v>99</v>
       </c>
@@ -1736,8 +1867,11 @@
         <v>8</v>
       </c>
       <c r="G47" s="9"/>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H47" s="10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A48" s="9" t="s">
         <v>99</v>
       </c>
@@ -1757,8 +1891,11 @@
         <v>7</v>
       </c>
       <c r="G48" s="9"/>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H48" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" s="9" t="s">
         <v>99</v>
       </c>
@@ -1778,8 +1915,11 @@
         <v>97</v>
       </c>
       <c r="G49" s="9"/>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H49" s="10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A50" s="9" t="s">
         <v>99</v>
       </c>
@@ -1801,8 +1941,11 @@
       <c r="G50" s="9" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H50" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A51" s="9" t="s">
         <v>99</v>
       </c>
@@ -1822,8 +1965,11 @@
         <v>8</v>
       </c>
       <c r="G51" s="9"/>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H51" s="10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A52" s="9" t="s">
         <v>99</v>
       </c>
@@ -1843,8 +1989,11 @@
         <v>31</v>
       </c>
       <c r="G52" s="9"/>
-    </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H52" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A53" s="9" t="s">
         <v>99</v>
       </c>
@@ -1864,8 +2013,11 @@
         <v>82</v>
       </c>
       <c r="G53" s="9"/>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H53" s="10" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A54" s="9" t="s">
         <v>99</v>
       </c>
@@ -1885,8 +2037,11 @@
         <v>8</v>
       </c>
       <c r="G54" s="9"/>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H54" s="10" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A55" s="9" t="s">
         <v>99</v>
       </c>
@@ -1906,8 +2061,11 @@
         <v>8</v>
       </c>
       <c r="G55" s="9"/>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H55" s="10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A56" s="9" t="s">
         <v>99</v>
       </c>
@@ -1927,6 +2085,9 @@
         <v>52</v>
       </c>
       <c r="G56" s="9"/>
+      <c r="H56" s="10" t="s">
+        <v>20</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>